<commit_message>
feat: add Chairus HOME shop, sync updated ROI and refresh multi-shop dashboard
</commit_message>
<xml_diff>
--- a/ROI记录表.xlsx
+++ b/ROI记录表.xlsx
@@ -2,41 +2,195 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="14400" windowHeight="12375" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日ROI记录" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00_ "/>
+  </numFmts>
+  <fonts count="23">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <charset val="134"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -45,12 +199,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="FF1E293B"/>
+        <bgColor rgb="FF1E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -60,37 +400,337 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </left>
       <right style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </right>
       <top style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -443,7 +1083,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -453,16 +1092,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E92"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>日期</t>
@@ -480,765 +1118,1220 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>HOME</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="16.5" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B2" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10.55</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>8.93</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="D5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="D7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="D10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="D11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>14.77</v>
+      </c>
+      <c r="D12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>14.81</v>
+      </c>
+      <c r="D13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="D14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="16.5" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="D15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="D16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="D17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="16.5" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="D19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="16.5" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>14.37</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="D20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="D21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="16.5" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>12.09</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="D22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="16.5" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="D23" s="4" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1">
+      <c r="A24" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="D24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="16.5" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D25" s="4" t="n"/>
+    </row>
+    <row r="26" ht="16.5" customHeight="1">
+      <c r="A26" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="16.5" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="D27" s="4" t="n"/>
+    </row>
+    <row r="28" ht="16.5" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="D28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="D29" s="4" t="n"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1">
+      <c r="A30" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="16.5" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="D31" s="4" t="n"/>
+    </row>
+    <row r="32" ht="16.5" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B32" s="3" t="n">
         <v>5.54</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C32" s="3" t="n">
         <v>5.12</v>
       </c>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B33" s="3" t="n">
         <v>2.67</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C33" s="3" t="n">
         <v>2.74</v>
       </c>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16.5" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B34" s="3" t="n">
         <v>3.99</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C34" s="3" t="n">
         <v>6.63</v>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16.5" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B35" s="3" t="n">
         <v>4.94</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C35" s="3" t="n">
         <v>13.34</v>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B36" s="3" t="n">
         <v>6.24</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C36" s="3" t="n">
         <v>8.58</v>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B37" s="3" t="n">
         <v>7.53</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C37" s="3" t="n">
         <v>5.84</v>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B38" s="3" t="n">
         <v>3.73</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C38" s="3" t="n">
         <v>7.01</v>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16.5" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B39" s="3" t="n">
         <v>7.47</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C39" s="3" t="n">
         <v>4.62</v>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B40" s="3" t="n">
         <v>9.42</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C40" s="3" t="n">
         <v>5.98</v>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16.5" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B41" s="3" t="n">
         <v>12.15</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C41" s="3" t="n">
         <v>9.640000000000001</v>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B42" s="3" t="n">
         <v>6.46</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C42" s="3" t="n">
         <v>12.16</v>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16.5" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B43" s="3" t="n">
         <v>8.98</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C43" s="3" t="n">
         <v>11.34</v>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16.5" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B44" s="3" t="n">
         <v>3.99</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C44" s="3" t="n">
         <v>7.81</v>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B45" s="3" t="n">
         <v>17.33</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C45" s="3" t="n">
         <v>10.3</v>
       </c>
-      <c r="D15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16.5" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B46" s="3" t="n">
         <v>12.3</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C46" s="3" t="n">
         <v>5.79</v>
       </c>
-      <c r="D16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16.5" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B47" s="3" t="n">
         <v>14.23</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C47" s="3" t="n">
         <v>10.39</v>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B48" s="3" t="n">
         <v>6.82</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C48" s="3" t="n">
         <v>4.71</v>
       </c>
-      <c r="D18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16.5" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B49" s="3" t="n">
         <v>4.67</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C49" s="3" t="n">
         <v>8.109999999999999</v>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="16.5" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>2026-07-19</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B50" s="3" t="n">
         <v>7.26</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C50" s="3" t="n">
         <v>6.38</v>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51" ht="16.5" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B51" s="3" t="n">
         <v>7.1</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C51" s="3" t="n">
         <v>7.6</v>
       </c>
-      <c r="D21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16.5" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B52" s="3" t="n">
         <v>5.1</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C52" s="3" t="n">
         <v>5.03</v>
       </c>
-      <c r="D22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B53" s="3" t="n">
         <v>4.43</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C53" s="3" t="n">
         <v>8.220000000000001</v>
       </c>
-      <c r="D23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16.5" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B54" s="3" t="n">
         <v>11.06</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C54" s="3" t="n">
         <v>3.02</v>
       </c>
-      <c r="D24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16.5" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B55" s="3" t="n">
         <v>9.85</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C55" s="3" t="n">
         <v>10.2</v>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16.5" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B56" s="3" t="n">
         <v>6.7</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C56" s="3" t="n">
         <v>4.38</v>
       </c>
-      <c r="D26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B57" s="3" t="n">
         <v>26.02</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C57" s="3" t="n">
         <v>8.19</v>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58" ht="16.5" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B58" s="3" t="n">
         <v>6.51</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C58" s="3" t="n">
         <v>7.06</v>
       </c>
-      <c r="D28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59" ht="16.5" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B59" s="3" t="n">
         <v>9.6</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C59" s="3" t="n">
         <v>13.1</v>
       </c>
-      <c r="D29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B60" s="3" t="n">
         <v>7.25</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C60" s="3" t="n">
         <v>7.9</v>
       </c>
-      <c r="D30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B61" s="3" t="n">
         <v>12.85</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C61" s="3" t="n">
         <v>11.47</v>
       </c>
-      <c r="D31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B62" s="3" t="n">
         <v>15.79</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C62" s="3" t="n">
         <v>9.49</v>
       </c>
-      <c r="D32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63" ht="16.5" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B63" s="3" t="n">
         <v>15.46</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C63" s="3" t="n">
         <v>5.67</v>
       </c>
-      <c r="D33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B64" s="3" t="n">
         <v>30.01</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C64" s="3" t="n">
         <v>15.35</v>
       </c>
-      <c r="D34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65" ht="16.5" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B65" s="3" t="n">
         <v>15.4</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C65" s="3" t="n">
         <v>6.16</v>
       </c>
-      <c r="D35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B66" s="3" t="n">
         <v>10.96</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C66" s="3" t="n">
         <v>6.28</v>
       </c>
-      <c r="D36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67" ht="16.5" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B67" s="3" t="n">
         <v>13.39</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C67" s="3" t="n">
         <v>5.66</v>
       </c>
-      <c r="D37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68" ht="16.5" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B68" s="3" t="n">
         <v>13.09</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C68" s="3" t="n">
         <v>11.56</v>
       </c>
-      <c r="D38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B69" s="3" t="n">
         <v>18.56</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C69" s="3" t="n">
         <v>10.65</v>
       </c>
-      <c r="D39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70" ht="16.5" customHeight="1">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B70" s="3" t="n">
         <v>8.27</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C70" s="3" t="n">
         <v>6.54</v>
       </c>
-      <c r="D40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71" ht="16.5" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B71" s="3" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C71" s="3" t="n">
         <v>4.55</v>
       </c>
-      <c r="D41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B72" s="3" t="n">
         <v>12.59</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C72" s="3" t="n">
         <v>6.12</v>
       </c>
-      <c r="D42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73" ht="16.5" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B73" s="3" t="n">
         <v>19.14</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="C73" s="3" t="n">
         <v>4.79</v>
       </c>
-      <c r="D43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="D73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74" ht="16.5" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B74" s="3" t="n">
         <v>9.91</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C74" s="3" t="n">
         <v>2.95</v>
       </c>
-      <c r="D44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75" ht="16.5" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B75" s="3" t="n">
         <v>10.94</v>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="C75" s="3" t="n">
         <v>5.54</v>
       </c>
-      <c r="D45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="D75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="16.5" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B76" s="3" t="n">
         <v>9.49</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C76" s="3" t="n">
         <v>6.88</v>
       </c>
-      <c r="D46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="D76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77" ht="16.5" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B77" s="3" t="n">
         <v>8.82</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="C77" s="3" t="n">
         <v>10.82</v>
       </c>
-      <c r="D47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78" ht="16.5" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B78" s="3" t="n">
         <v>9.25</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C78" s="3" t="n">
         <v>7.06</v>
       </c>
-      <c r="D48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79" ht="16.5" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B79" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C79" s="3" t="n">
         <v>8.32</v>
       </c>
-      <c r="D49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80" ht="16.5" customHeight="1">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B80" s="3" t="n">
         <v>7.01</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C80" s="3" t="n">
         <v>4.36</v>
       </c>
-      <c r="D50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="D80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81" ht="16.5" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B81" s="3" t="n">
         <v>20.11</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C81" s="3" t="n">
         <v>8.449999999999999</v>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="D81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82" ht="16.5" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n">
+      <c r="B82" s="3" t="n">
         <v>10.44</v>
       </c>
-      <c r="C52" s="3" t="n">
+      <c r="C82" s="3" t="n">
         <v>5.98</v>
       </c>
-      <c r="D52" s="4" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="D82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83" ht="16.5" customHeight="1">
+      <c r="A83" s="6" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B83" s="3" t="n">
         <v>19.11</v>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="C83" s="3" t="n">
         <v>4.1</v>
       </c>
-      <c r="D53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="D83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84" ht="16.5" customHeight="1">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B84" s="3" t="n">
         <v>9.56</v>
       </c>
-      <c r="C54" s="3" t="n">
+      <c r="C84" s="3" t="n">
         <v>6.02</v>
       </c>
-      <c r="D54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="D84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85" ht="16.5" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B55" s="3" t="n">
+      <c r="B85" s="3" t="n">
         <v>16.31</v>
       </c>
-      <c r="C55" s="3" t="n">
+      <c r="C85" s="3" t="n">
         <v>10.25</v>
       </c>
-      <c r="D55" s="4" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86" ht="16.5" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="C86" t="n">
+        <v>5.18</v>
+      </c>
+    </row>
+    <row r="87" ht="16.5" customHeight="1">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="C87" t="n">
+        <v>5.79</v>
+      </c>
+    </row>
+    <row r="88" ht="16.5" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>13.36</v>
+      </c>
+      <c r="C88" t="n">
+        <v>8.76</v>
+      </c>
+    </row>
+    <row r="89" ht="16.5" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C89" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="90" ht="16.5" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>14.89</v>
+      </c>
+      <c r="C90" t="n">
+        <v>12.27</v>
+      </c>
+    </row>
+    <row r="91" ht="16.5" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="C91" t="n">
+        <v>7.55</v>
+      </c>
+    </row>
+    <row r="92" ht="16.5" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="C92" t="n">
+        <v>6.18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>